<commit_message>
Add Main5 data, analysis and full dataset analysis
</commit_message>
<xml_diff>
--- a/Utterances/Annotation_Main/Main5/Main5_Katja.xlsx
+++ b/Utterances/Annotation_Main/Main5/Main5_Katja.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\katjam\Dropbox\Doktorat\ParlaMint\Sentiment_annotation-speeches\Annotation_Main\Main5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\katjam\Dropbox\Doktorat\ParlaMint\Sentiment_annotation\Utterances\Annotation_Main\Main5\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="14235"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="474">
   <si>
     <t>ID</t>
   </si>
@@ -1266,24 +1266,12 @@
     <t>There are some positive points in this, but the speech seems to lean more towards negative. Could also be M_Positive</t>
   </si>
   <si>
-    <t>Overall very negative in tone, but the sentiment shifts at several points into positive. So, would have a hard time annotating this as purely negative.</t>
-  </si>
-  <si>
     <t>Not a lot of context, but could also be N_Negative</t>
   </si>
   <si>
-    <t xml:space="preserve">Very procedural, just outlining the amendments that were/were not supported. </t>
-  </si>
-  <si>
     <t>Chair speaking, but here we have a very positive speech in the first part, the second is moving onto the agenda items for the day. But overall, I would say it is positive.</t>
   </si>
   <si>
-    <t xml:space="preserve">Could also be entirely Negative, but due to the first very positive part, I will </t>
-  </si>
-  <si>
-    <t>This one could also be N_Neutral, but due to two specific words, I do not this this is neutral. But also, not a lot of context is given..</t>
-  </si>
-  <si>
     <t>This to me is positive throughout, at points a bit more weak, as the speaker outlines the new and improved points.</t>
   </si>
   <si>
@@ -1311,9 +1299,6 @@
     <t>Ok, this is direct Negative, there is nothing neutral about that</t>
   </si>
   <si>
-    <t>Could also be P_Neutral.</t>
-  </si>
-  <si>
     <t>They will support the bill, and at the end there is a positive statement right at the end. I do not know, it is very negative in tone, so it could be Negative.</t>
   </si>
   <si>
@@ -1323,35 +1308,146 @@
     <t>Weak negative</t>
   </si>
   <si>
-    <t xml:space="preserve">While the first part just describes the amendment and what it requires, the second part is actually quite negative.  </t>
-  </si>
-  <si>
     <t>Charged and slightly accusatory questions.</t>
   </si>
   <si>
     <t>Second part is very negative, but in the first part the speaker emphasises some positive aspects that he is supporting. So not entirely negative. But if we only go on the overall tone, then it could also be Negative.</t>
   </si>
   <si>
-    <t>Defensive, with slight positive points throughout. But the tone is very negative.</t>
-  </si>
-  <si>
     <t>Maybe not the strongest negative sentiment ever, but still negative.</t>
   </si>
   <si>
-    <t xml:space="preserve">Accusatory on one hand and defensive on the other. </t>
-  </si>
-  <si>
     <t>Negative connotation, warning</t>
   </si>
   <si>
     <t>????</t>
+  </si>
+  <si>
+    <t>Very procedural, just outlining the amendments that were/were not supported. </t>
+  </si>
+  <si>
+    <t>While the first part just describes the amendment and what it requires, the second part is actually quite negative.  </t>
+  </si>
+  <si>
+    <t>Accusatory on one hand and defensive on the other. </t>
+  </si>
+  <si>
+    <t>The speaker and his PS supports the law and the amendments, however, the the second part of the speech is very negative. Could also be M_Positive, should we take this second part as an explanation to better sell the amendments.</t>
+  </si>
+  <si>
+    <t>The middle of the speech is somewhat negative, but the rest of the speech is supportive and in positive tone</t>
+  </si>
+  <si>
+    <t>Consistently negative speech, maybe not the strongest negative, but still the speaker explains why these points are not okay (with somewhat harsh words at time)</t>
+  </si>
+  <si>
+    <t>Relatively neutral speech.</t>
+  </si>
+  <si>
+    <t>Slightly defensive explanation.</t>
+  </si>
+  <si>
+    <t>Could also be N_Neutral, should this be considered a warning, but there is not enough context.</t>
+  </si>
+  <si>
+    <t>Negative connotation and charged questions.</t>
+  </si>
+  <si>
+    <t>Explanation, with positive connotation at the end, but mostly defensive and negative in the first part of the speech.</t>
+  </si>
+  <si>
+    <t>Could also be Positive, as the negative insertions serve as additional emphasis why the </t>
+  </si>
+  <si>
+    <t>Negative topic, presentation of the bill in current form, with the support of it. Not sure of the sentiment behind it, seems fairly neutral.</t>
+  </si>
+  <si>
+    <t>The end seems slightly negative in connotation. But could also be P_Neutral.</t>
+  </si>
+  <si>
+    <t>Warning, but procedural. Could also be Negative.</t>
+  </si>
+  <si>
+    <t>I do not sense a particular sentiment here, the whole speech seems rather neutral. </t>
+  </si>
+  <si>
+    <t>This one is interesting - the speech is mostly positive (given a relatively negative topic) and the whole thing ends with a support the decision that the proposal is not suitable for further processing.</t>
+  </si>
+  <si>
+    <t>Sarcastic and accusatory.</t>
+  </si>
+  <si>
+    <t>Question to MP, seems relatively neutral (as there is not a lot of context with this one).</t>
+  </si>
+  <si>
+    <t>Charged question, definitely not neutral. </t>
+  </si>
+  <si>
+    <t>The speaker outlines the (negative) opinion that they have given. Given this, it could also be Negative</t>
+  </si>
+  <si>
+    <t>The middle part of speech is a bit less positive (justification and describing positive changes), but overall, the speech is positive.</t>
+  </si>
+  <si>
+    <t>Weird sentence, seems slightly negative.</t>
+  </si>
+  <si>
+    <t>This one could also be N_Neutral, but due to two specific words, I do not think this this is neutral. But also, not a lot of context is given..</t>
+  </si>
+  <si>
+    <t>At points this speech does contain some positive points (though weak).</t>
+  </si>
+  <si>
+    <t>Could also be N_Neutral if we take this just as a warning. But given the “in še 4 sekunde”, I think this is just pure negative.</t>
+  </si>
+  <si>
+    <t>Call to keep one of the articles in the bill, seems to be slightly negative.</t>
+  </si>
+  <si>
+    <t>Might not be the strongest negative, but seems to be consistently negative.</t>
+  </si>
+  <si>
+    <t>Some negative critique on the media covering, but overall very positive otherwise.</t>
+  </si>
+  <si>
+    <t>Some positive points in the speech, but otherwise negative</t>
+  </si>
+  <si>
+    <t>Overall negative with some positive interventions. Could also be directly Negative (as the second part is very negative)</t>
+  </si>
+  <si>
+    <t>Negative topics, but just an explanation of todays procedures and outcomes, does not carry any explicit sentiment.</t>
+  </si>
+  <si>
+    <t>Second part is defensive, and overall negative speech.</t>
+  </si>
+  <si>
+    <t>The speaker expresses support for the changes, however is aware of the larger issues and the fact that the changes will bring only smaller positive changes. Most of the speech however, is relatively negative.</t>
+  </si>
+  <si>
+    <t>Weak positive, reply to a question. </t>
+  </si>
+  <si>
+    <t>Could also be Negative</t>
+  </si>
+  <si>
+    <t>Could also be entirely Negative, but due to the first very positive part, I think it is Mixed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overall very negative in tone, but the sentiment shifts at several points into positive. So, would have a hard time annotating this as purely negative. </t>
+  </si>
+  <si>
+    <t>Defensive and negative.</t>
+  </si>
+  <si>
+    <t>Could also be N_Neutral.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1364,6 +1460,27 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -1374,7 +1491,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1417,7 +1534,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1431,14 +1548,38 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Navadno" xfId="0" builtinId="0"/>
@@ -1741,8 +1882,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G201"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H201"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="44.42578125" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="142.140625" style="3" customWidth="1"/>
@@ -1762,7 +1903,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1775,16 +1916,17 @@
         <v>406</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s">
-        <v>408</v>
-      </c>
+      <c r="C2" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D2" s="9"/>
       <c r="F2" t="b">
         <v>1</v>
       </c>
@@ -1799,10 +1941,10 @@
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" t="s">
-        <v>412</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="C3" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>413</v>
       </c>
       <c r="F3" t="b">
@@ -1819,9 +1961,10 @@
       <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="7" t="s">
         <v>407</v>
       </c>
+      <c r="D4" s="9"/>
       <c r="F4" t="b">
         <v>0</v>
       </c>
@@ -1829,16 +1972,17 @@
         <v>409</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>408</v>
-      </c>
+      <c r="C5" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D5" s="9"/>
       <c r="F5" t="b">
         <v>1</v>
       </c>
@@ -1846,16 +1990,17 @@
         <v>410</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C6" t="s">
-        <v>408</v>
-      </c>
+      <c r="C6" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D6" s="9"/>
       <c r="F6" t="b">
         <v>1</v>
       </c>
@@ -1870,10 +2015,10 @@
       <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="11" t="s">
         <v>411</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="12" t="s">
         <v>414</v>
       </c>
       <c r="E7" s="6" t="b">
@@ -1893,11 +2038,11 @@
       <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="11" t="s">
         <v>411</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>415</v>
+      <c r="D8" s="12" t="s">
+        <v>471</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -1910,14 +2055,14 @@
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="8" t="s">
-        <v>408</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>416</v>
+      <c r="C9" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>415</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -1930,9 +2075,10 @@
       <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>412</v>
-      </c>
+      <c r="C10" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D10" s="9"/>
       <c r="F10" t="b">
         <v>0</v>
       </c>
@@ -1944,9 +2090,10 @@
       <c r="B11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C11" t="s">
-        <v>408</v>
-      </c>
+      <c r="C11" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D11" s="9"/>
       <c r="F11" t="b">
         <v>1</v>
       </c>
@@ -1958,9 +2105,10 @@
       <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C12" t="s">
-        <v>412</v>
-      </c>
+      <c r="C12" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D12" s="9"/>
       <c r="F12" t="b">
         <v>0</v>
       </c>
@@ -1972,38 +2120,40 @@
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C13" t="s">
-        <v>408</v>
-      </c>
+      <c r="C13" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D13" s="9"/>
       <c r="F13" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="8" t="s">
-        <v>408</v>
-      </c>
-      <c r="D14" s="7"/>
+      <c r="C14" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D14" s="9"/>
       <c r="F14" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C15" t="s">
-        <v>408</v>
-      </c>
+      <c r="C15" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D15" s="9"/>
       <c r="F15" t="b">
         <v>1</v>
       </c>
@@ -2015,9 +2165,10 @@
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C16" t="s">
-        <v>408</v>
-      </c>
+      <c r="C16" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D16" s="9"/>
       <c r="F16" t="b">
         <v>0</v>
       </c>
@@ -2029,51 +2180,55 @@
       <c r="B17" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C17" t="s">
-        <v>412</v>
-      </c>
+      <c r="C17" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D17" s="9"/>
       <c r="F17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>38</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C18" t="s">
-        <v>408</v>
-      </c>
+      <c r="C18" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D18" s="9"/>
       <c r="F18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C19" t="s">
-        <v>408</v>
-      </c>
+      <c r="C19" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D19" s="9"/>
       <c r="F19" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C20" t="s">
-        <v>408</v>
-      </c>
+      <c r="C20" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D20" s="9"/>
       <c r="F20" t="b">
         <v>1</v>
       </c>
@@ -2085,9 +2240,10 @@
       <c r="B21" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C21" t="s">
-        <v>412</v>
-      </c>
+      <c r="C21" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D21" s="9"/>
       <c r="F21" t="b">
         <v>0</v>
       </c>
@@ -2099,9 +2255,10 @@
       <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C22" t="s">
-        <v>408</v>
-      </c>
+      <c r="C22" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D22" s="9"/>
       <c r="F22" t="b">
         <v>0</v>
       </c>
@@ -2113,11 +2270,11 @@
       <c r="B23" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C23" t="s">
-        <v>408</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>417</v>
+      <c r="C23" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>434</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -2130,9 +2287,10 @@
       <c r="B24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="C24" t="s">
-        <v>408</v>
-      </c>
+      <c r="C24" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D24" s="9"/>
       <c r="F24" t="b">
         <v>1</v>
       </c>
@@ -2141,43 +2299,45 @@
       <c r="A25" t="s">
         <v>52</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>418</v>
+      <c r="D25" s="10" t="s">
+        <v>416</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>54</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C26" t="s">
-        <v>408</v>
-      </c>
+      <c r="C26" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D26" s="9"/>
       <c r="F26" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>56</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="C27" t="s">
-        <v>408</v>
-      </c>
+      <c r="C27" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D27" s="9"/>
       <c r="F27" t="b">
         <v>1</v>
       </c>
@@ -2186,28 +2346,29 @@
       <c r="A28" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="7" t="s">
+      <c r="B28" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C28" s="8" t="s">
-        <v>412</v>
-      </c>
-      <c r="D28" s="7"/>
-      <c r="E28" s="8"/>
+      <c r="C28" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D28" s="9"/>
+      <c r="E28" s="6"/>
       <c r="F28" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>60</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C29" t="s">
-        <v>408</v>
-      </c>
+      <c r="C29" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D29" s="9"/>
       <c r="F29" t="b">
         <v>1</v>
       </c>
@@ -2219,9 +2380,10 @@
       <c r="B30" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C30" t="s">
-        <v>412</v>
-      </c>
+      <c r="C30" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D30" s="9"/>
       <c r="F30" t="b">
         <v>0</v>
       </c>
@@ -2233,11 +2395,11 @@
       <c r="B31" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="D31" s="3" t="s">
-        <v>419</v>
+      <c r="D31" s="10" t="s">
+        <v>470</v>
       </c>
       <c r="F31" t="b">
         <v>0</v>
@@ -2250,9 +2412,10 @@
       <c r="B32" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="7" t="s">
         <v>407</v>
       </c>
+      <c r="D32" s="9"/>
       <c r="F32" t="b">
         <v>0</v>
       </c>
@@ -2264,11 +2427,11 @@
       <c r="B33" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="7" t="s">
         <v>407</v>
       </c>
-      <c r="D33" s="3" t="s">
-        <v>421</v>
+      <c r="D33" s="10" t="s">
+        <v>417</v>
       </c>
       <c r="F33" t="b">
         <v>0</v>
@@ -2281,11 +2444,11 @@
       <c r="B34" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>422</v>
+      <c r="C34" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>418</v>
       </c>
       <c r="E34" s="6" t="b">
         <v>1</v>
@@ -2301,26 +2464,27 @@
       <c r="B35" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C35" t="s">
-        <v>412</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>423</v>
+      <c r="C35" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>419</v>
       </c>
       <c r="F35" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>74</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="C36" t="s">
-        <v>408</v>
-      </c>
+      <c r="C36" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D36" s="9"/>
       <c r="F36" t="b">
         <v>1</v>
       </c>
@@ -2332,11 +2496,11 @@
       <c r="B37" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="D37" s="3" t="s">
-        <v>424</v>
+      <c r="D37" s="10" t="s">
+        <v>420</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
@@ -2349,37 +2513,40 @@
       <c r="B38" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C38" t="s">
-        <v>408</v>
-      </c>
+      <c r="C38" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D38" s="9"/>
       <c r="F38" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>80</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="C39" t="s">
-        <v>408</v>
-      </c>
+      <c r="C39" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D39" s="9"/>
       <c r="F39" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>82</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="C40" t="s">
-        <v>408</v>
-      </c>
+      <c r="C40" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D40" s="9"/>
       <c r="F40" t="b">
         <v>1</v>
       </c>
@@ -2391,11 +2558,11 @@
       <c r="B41" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="11" t="s">
         <v>409</v>
       </c>
-      <c r="D41" s="5" t="s">
-        <v>425</v>
+      <c r="D41" s="12" t="s">
+        <v>421</v>
       </c>
       <c r="E41" s="6" t="b">
         <v>1</v>
@@ -2411,9 +2578,10 @@
       <c r="B42" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C42" t="s">
-        <v>408</v>
-      </c>
+      <c r="C42" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D42" s="9"/>
       <c r="F42" t="b">
         <v>1</v>
       </c>
@@ -2425,11 +2593,11 @@
       <c r="B43" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="C43" t="s">
-        <v>408</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>426</v>
+      <c r="C43" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>422</v>
       </c>
       <c r="F43" t="b">
         <v>0</v>
@@ -2442,11 +2610,11 @@
       <c r="B44" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="11" t="s">
         <v>411</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>428</v>
+      <c r="D44" s="12" t="s">
+        <v>424</v>
       </c>
       <c r="E44" s="6" t="b">
         <v>1</v>
@@ -2462,11 +2630,11 @@
       <c r="B45" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C45" t="s">
-        <v>408</v>
-      </c>
-      <c r="D45" s="3" t="s">
-        <v>427</v>
+      <c r="C45" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>423</v>
       </c>
       <c r="F45" t="b">
         <v>0</v>
@@ -2479,9 +2647,10 @@
       <c r="B46" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="C46" t="s">
-        <v>412</v>
-      </c>
+      <c r="C46" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D46" s="9"/>
       <c r="F46" t="b">
         <v>0</v>
       </c>
@@ -2493,23 +2662,25 @@
       <c r="B47" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C47" t="s">
-        <v>408</v>
-      </c>
+      <c r="C47" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D47" s="9"/>
       <c r="F47" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>98</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C48" t="s">
-        <v>408</v>
-      </c>
+      <c r="C48" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D48" s="9"/>
       <c r="F48" t="b">
         <v>1</v>
       </c>
@@ -2521,26 +2692,27 @@
       <c r="B49" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C49" t="s">
-        <v>412</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>429</v>
+      <c r="C49" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>425</v>
       </c>
       <c r="F49" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>102</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C50" t="s">
-        <v>408</v>
-      </c>
+      <c r="C50" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D50" s="9"/>
       <c r="F50" t="b">
         <v>1</v>
       </c>
@@ -2552,9 +2724,10 @@
       <c r="B51" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="C51" t="s">
-        <v>408</v>
-      </c>
+      <c r="C51" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D51" s="9"/>
       <c r="F51" t="b">
         <v>1</v>
       </c>
@@ -2566,9 +2739,10 @@
       <c r="B52" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="C52" t="s">
-        <v>412</v>
-      </c>
+      <c r="C52" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D52" s="9"/>
       <c r="F52" t="b">
         <v>0</v>
       </c>
@@ -2580,11 +2754,11 @@
       <c r="B53" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="C53" s="6" t="s">
-        <v>409</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>430</v>
+      <c r="C53" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="D53" s="12" t="s">
+        <v>473</v>
       </c>
       <c r="E53" s="6" t="b">
         <v>1</v>
@@ -2600,29 +2774,29 @@
       <c r="B54" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C54" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D54" s="5" t="s">
-        <v>433</v>
+      <c r="C54" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>428</v>
       </c>
       <c r="E54" s="6"/>
       <c r="F54" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>112</v>
       </c>
-      <c r="B55" s="7" t="s">
+      <c r="B55" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C55" s="8" t="s">
-        <v>408</v>
-      </c>
-      <c r="D55" s="7"/>
-      <c r="E55" s="8"/>
+      <c r="C55" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D55" s="9"/>
+      <c r="E55" s="6"/>
       <c r="F55" t="b">
         <v>1</v>
       </c>
@@ -2631,16 +2805,16 @@
       <c r="A56" t="s">
         <v>114</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B56" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="C56" s="8" t="s">
+      <c r="C56" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="D56" s="7" t="s">
-        <v>431</v>
-      </c>
-      <c r="E56" s="8" t="b">
+      <c r="D56" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="E56" s="6" t="b">
         <v>1</v>
       </c>
       <c r="F56" t="b">
@@ -2651,16 +2825,16 @@
       <c r="A57" t="s">
         <v>116</v>
       </c>
-      <c r="B57" s="7" t="s">
+      <c r="B57" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="C57" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="D57" s="7" t="s">
-        <v>432</v>
-      </c>
-      <c r="E57" s="8"/>
+      <c r="D57" s="10" t="s">
+        <v>427</v>
+      </c>
+      <c r="E57" s="6"/>
       <c r="F57" t="b">
         <v>1</v>
       </c>
@@ -2672,11 +2846,11 @@
       <c r="B58" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C58" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D58" s="5" t="s">
-        <v>434</v>
+      <c r="C58" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>435</v>
       </c>
       <c r="E58" s="6"/>
       <c r="F58" t="b">
@@ -2690,23 +2864,25 @@
       <c r="B59" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C59" t="s">
-        <v>412</v>
-      </c>
+      <c r="C59" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D59" s="9"/>
       <c r="F59" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>122</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C60" t="s">
-        <v>408</v>
-      </c>
+      <c r="C60" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D60" s="9"/>
       <c r="F60" t="b">
         <v>1</v>
       </c>
@@ -2718,11 +2894,11 @@
       <c r="B61" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="C61" t="s">
-        <v>412</v>
-      </c>
-      <c r="D61" s="3" t="s">
-        <v>438</v>
+      <c r="C61" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D61" s="10" t="s">
+        <v>431</v>
       </c>
       <c r="F61" t="b">
         <v>0</v>
@@ -2735,23 +2911,25 @@
       <c r="B62" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="C62" t="s">
-        <v>408</v>
-      </c>
+      <c r="C62" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D62" s="9"/>
       <c r="F62" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>128</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C63" t="s">
-        <v>408</v>
-      </c>
+      <c r="C63" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D63" s="9"/>
       <c r="F63" t="b">
         <v>1</v>
       </c>
@@ -2763,40 +2941,42 @@
       <c r="B64" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C64" t="s">
-        <v>412</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>435</v>
+      <c r="C64" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>429</v>
       </c>
       <c r="F64" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>132</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="C65" t="s">
-        <v>408</v>
-      </c>
+      <c r="C65" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D65" s="9"/>
       <c r="F65" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>134</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="C66" t="s">
-        <v>408</v>
-      </c>
+      <c r="C66" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D66" s="9"/>
       <c r="F66" t="b">
         <v>1</v>
       </c>
@@ -2808,11 +2988,11 @@
       <c r="B67" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C67" t="s">
+      <c r="C67" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="D67" s="3" t="s">
-        <v>436</v>
+      <c r="D67" s="10" t="s">
+        <v>430</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
@@ -2825,9 +3005,10 @@
       <c r="B68" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="C68" t="s">
-        <v>408</v>
-      </c>
+      <c r="C68" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D68" s="9"/>
       <c r="F68" t="b">
         <v>1</v>
       </c>
@@ -2839,11 +3020,11 @@
       <c r="B69" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C69" s="6" t="s">
-        <v>411</v>
-      </c>
-      <c r="D69" s="5" t="s">
-        <v>437</v>
+      <c r="C69" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>472</v>
       </c>
       <c r="E69" s="6" t="b">
         <v>1</v>
@@ -2859,9 +3040,10 @@
       <c r="B70" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="C70" t="s">
-        <v>412</v>
-      </c>
+      <c r="C70" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D70" s="9"/>
       <c r="F70" t="b">
         <v>0</v>
       </c>
@@ -2873,23 +3055,25 @@
       <c r="B71" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C71" t="s">
-        <v>412</v>
-      </c>
+      <c r="C71" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D71" s="9"/>
       <c r="F71" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>146</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="C72" t="s">
-        <v>412</v>
-      </c>
+      <c r="C72" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D72" s="9"/>
       <c r="F72" t="b">
         <v>1</v>
       </c>
@@ -2901,9 +3085,10 @@
       <c r="B73" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C73" t="s">
-        <v>412</v>
-      </c>
+      <c r="C73" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D73" s="9"/>
       <c r="F73" t="b">
         <v>0</v>
       </c>
@@ -2915,9 +3100,10 @@
       <c r="B74" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C74" t="s">
-        <v>408</v>
-      </c>
+      <c r="C74" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D74" s="9"/>
       <c r="F74" t="b">
         <v>0</v>
       </c>
@@ -2929,9 +3115,10 @@
       <c r="B75" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C75" t="s">
-        <v>412</v>
-      </c>
+      <c r="C75" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D75" s="9"/>
       <c r="F75" t="b">
         <v>0</v>
       </c>
@@ -2940,14 +3127,14 @@
       <c r="A76" t="s">
         <v>154</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B76" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C76" s="8" t="s">
+      <c r="C76" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="D76" s="7"/>
-      <c r="E76" s="8"/>
+      <c r="D76" s="9"/>
+      <c r="E76" s="6"/>
       <c r="F76" t="b">
         <v>1</v>
       </c>
@@ -2959,11 +3146,11 @@
       <c r="B77" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="C77" t="s">
-        <v>412</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>439</v>
+      <c r="C77" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D77" s="10" t="s">
+        <v>436</v>
       </c>
       <c r="F77" t="b">
         <v>0</v>
@@ -2976,11 +3163,11 @@
       <c r="B78" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="C78" s="6" t="s">
+      <c r="C78" s="11" t="s">
         <v>411</v>
       </c>
-      <c r="D78" s="5" t="s">
-        <v>441</v>
+      <c r="D78" s="12" t="s">
+        <v>433</v>
       </c>
       <c r="E78" s="6" t="b">
         <v>1</v>
@@ -2996,9 +3183,10 @@
       <c r="B79" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C79" s="7" t="s">
         <v>411</v>
       </c>
+      <c r="D79" s="9"/>
       <c r="E79" t="b">
         <v>1</v>
       </c>
@@ -3013,65 +3201,70 @@
       <c r="B80" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="C80" t="s">
-        <v>408</v>
-      </c>
+      <c r="C80" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D80" s="9"/>
       <c r="F80" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>164</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C81" t="s">
-        <v>408</v>
-      </c>
+      <c r="C81" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D81" s="9"/>
       <c r="F81" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>166</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C82" t="s">
-        <v>408</v>
-      </c>
+      <c r="C82" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D82" s="9"/>
       <c r="F82" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>168</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="C83" t="s">
-        <v>408</v>
-      </c>
+      <c r="C83" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D83" s="9"/>
       <c r="F83" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>170</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C84" t="s">
-        <v>408</v>
-      </c>
+      <c r="C84" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D84" s="9"/>
       <c r="F84" t="b">
         <v>1</v>
       </c>
@@ -3083,11 +3276,11 @@
       <c r="B85" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="C85" t="s">
+      <c r="C85" s="7" t="s">
         <v>409</v>
       </c>
-      <c r="D85" s="3" t="s">
-        <v>440</v>
+      <c r="D85" s="10" t="s">
+        <v>432</v>
       </c>
       <c r="F85" t="b">
         <v>1</v>
@@ -3100,6 +3293,12 @@
       <c r="B86" s="3" t="s">
         <v>175</v>
       </c>
+      <c r="C86" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D86" s="10" t="s">
+        <v>437</v>
+      </c>
       <c r="F86" t="b">
         <v>0</v>
       </c>
@@ -3111,6 +3310,12 @@
       <c r="B87" s="3" t="s">
         <v>177</v>
       </c>
+      <c r="C87" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="D87" s="10" t="s">
+        <v>438</v>
+      </c>
       <c r="F87" t="b">
         <v>0</v>
       </c>
@@ -3122,6 +3327,12 @@
       <c r="B88" s="3" t="s">
         <v>179</v>
       </c>
+      <c r="C88" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D88" s="10" t="s">
+        <v>439</v>
+      </c>
       <c r="F88" t="b">
         <v>0</v>
       </c>
@@ -3133,6 +3344,10 @@
       <c r="B89" s="3" t="s">
         <v>181</v>
       </c>
+      <c r="C89" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D89" s="9"/>
       <c r="F89" t="b">
         <v>1</v>
       </c>
@@ -3144,6 +3359,12 @@
       <c r="B90" s="3" t="s">
         <v>183</v>
       </c>
+      <c r="C90" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D90" s="10" t="s">
+        <v>440</v>
+      </c>
       <c r="F90" t="b">
         <v>0</v>
       </c>
@@ -3155,28 +3376,42 @@
       <c r="B91" s="3" t="s">
         <v>185</v>
       </c>
+      <c r="C91" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D91" s="10" t="s">
+        <v>441</v>
+      </c>
       <c r="F91" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>186</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>187</v>
       </c>
+      <c r="C92" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D92" s="9"/>
       <c r="F92" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>188</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>189</v>
       </c>
+      <c r="C93" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D93" s="9"/>
       <c r="F93" t="b">
         <v>1</v>
       </c>
@@ -3188,38 +3423,56 @@
       <c r="B94" s="3" t="s">
         <v>191</v>
       </c>
+      <c r="C94" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D94" s="9"/>
       <c r="F94" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>192</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>193</v>
       </c>
+      <c r="C95" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D95" s="9"/>
       <c r="F95" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>194</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>195</v>
       </c>
+      <c r="C96" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D96" s="9"/>
       <c r="F96" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>196</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>197</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D97" s="10" t="s">
+        <v>442</v>
       </c>
       <c r="F97" t="b">
         <v>1</v>
@@ -3232,6 +3485,10 @@
       <c r="B98" s="3" t="s">
         <v>199</v>
       </c>
+      <c r="C98" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D98" s="9"/>
       <c r="F98" t="b">
         <v>1</v>
       </c>
@@ -3243,6 +3500,12 @@
       <c r="B99" s="3" t="s">
         <v>201</v>
       </c>
+      <c r="C99" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D99" s="10" t="s">
+        <v>443</v>
+      </c>
       <c r="F99" t="b">
         <v>0</v>
       </c>
@@ -3251,9 +3514,16 @@
       <c r="A100" t="s">
         <v>202</v>
       </c>
-      <c r="B100" s="3" t="s">
+      <c r="B100" s="5" t="s">
         <v>203</v>
       </c>
+      <c r="C100" s="11" t="s">
+        <v>411</v>
+      </c>
+      <c r="D100" s="12" t="s">
+        <v>444</v>
+      </c>
+      <c r="E100" s="6"/>
       <c r="F100" t="b">
         <v>0</v>
       </c>
@@ -3265,28 +3535,42 @@
       <c r="B101" s="3" t="s">
         <v>205</v>
       </c>
+      <c r="C101" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="D101" s="10" t="s">
+        <v>445</v>
+      </c>
       <c r="F101" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>206</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>207</v>
       </c>
+      <c r="C102" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D102" s="9"/>
       <c r="F102" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>208</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>209</v>
       </c>
+      <c r="C103" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D103" s="9"/>
       <c r="F103" t="b">
         <v>1</v>
       </c>
@@ -3298,6 +3582,10 @@
       <c r="B104" s="3" t="s">
         <v>211</v>
       </c>
+      <c r="C104" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D104" s="9"/>
       <c r="F104" t="b">
         <v>1</v>
       </c>
@@ -3306,42 +3594,61 @@
       <c r="A105" t="s">
         <v>212</v>
       </c>
-      <c r="B105" s="3" t="s">
+      <c r="B105" s="5" t="s">
         <v>213</v>
       </c>
+      <c r="C105" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="D105" s="12" t="s">
+        <v>446</v>
+      </c>
+      <c r="E105" s="6"/>
       <c r="F105" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>214</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>215</v>
       </c>
+      <c r="C106" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D106" s="9"/>
       <c r="F106" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>216</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>217</v>
       </c>
+      <c r="C107" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D107" s="9"/>
       <c r="F107" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>218</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>219</v>
       </c>
+      <c r="C108" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D108" s="9"/>
       <c r="F108" t="b">
         <v>1</v>
       </c>
@@ -3353,17 +3660,27 @@
       <c r="B109" s="3" t="s">
         <v>221</v>
       </c>
+      <c r="C109" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D109" s="10" t="s">
+        <v>447</v>
+      </c>
       <c r="F109" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>222</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>223</v>
       </c>
+      <c r="C110" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D110" s="9"/>
       <c r="F110" t="b">
         <v>1</v>
       </c>
@@ -3375,17 +3692,25 @@
       <c r="B111" s="3" t="s">
         <v>225</v>
       </c>
+      <c r="C111" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D111" s="9"/>
       <c r="F111" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>226</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>227</v>
       </c>
+      <c r="C112" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D112" s="9"/>
       <c r="F112" t="b">
         <v>1</v>
       </c>
@@ -3397,6 +3722,10 @@
       <c r="B113" s="3" t="s">
         <v>229</v>
       </c>
+      <c r="C113" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D113" s="9"/>
       <c r="F113" t="b">
         <v>0</v>
       </c>
@@ -3408,17 +3737,25 @@
       <c r="B114" s="3" t="s">
         <v>231</v>
       </c>
+      <c r="C114" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D114" s="9"/>
       <c r="F114" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>232</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>233</v>
       </c>
+      <c r="C115" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D115" s="9"/>
       <c r="F115" t="b">
         <v>0</v>
       </c>
@@ -3430,17 +3767,28 @@
       <c r="B116" s="3" t="s">
         <v>235</v>
       </c>
+      <c r="C116" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D116" s="9"/>
       <c r="F116" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>236</v>
       </c>
-      <c r="B117" s="3" t="s">
+      <c r="B117" s="5" t="s">
         <v>237</v>
       </c>
+      <c r="C117" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="D117" s="12" t="s">
+        <v>448</v>
+      </c>
+      <c r="E117" s="6"/>
       <c r="F117" t="b">
         <v>1</v>
       </c>
@@ -3452,17 +3800,25 @@
       <c r="B118" s="3" t="s">
         <v>239</v>
       </c>
+      <c r="C118" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D118" s="9"/>
       <c r="F118" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>240</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>241</v>
       </c>
+      <c r="C119" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D119" s="9"/>
       <c r="F119" t="b">
         <v>1</v>
       </c>
@@ -3471,31 +3827,44 @@
       <c r="A120" t="s">
         <v>242</v>
       </c>
-      <c r="B120" s="3" t="s">
+      <c r="B120" s="5" t="s">
         <v>243</v>
       </c>
+      <c r="C120" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D120" s="13"/>
+      <c r="E120" s="6"/>
       <c r="F120" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>244</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>245</v>
       </c>
+      <c r="C121" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D121" s="9"/>
       <c r="F121" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>246</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>247</v>
       </c>
+      <c r="C122" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D122" s="9"/>
       <c r="F122" t="b">
         <v>1</v>
       </c>
@@ -3507,28 +3876,40 @@
       <c r="B123" s="3" t="s">
         <v>249</v>
       </c>
+      <c r="C123" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D123" s="9"/>
       <c r="F123" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>250</v>
       </c>
       <c r="B124" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="C124" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D124" s="9"/>
       <c r="F124" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>252</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>253</v>
       </c>
+      <c r="C125" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D125" s="9"/>
       <c r="F125" t="b">
         <v>1</v>
       </c>
@@ -3540,17 +3921,25 @@
       <c r="B126" s="3" t="s">
         <v>255</v>
       </c>
+      <c r="C126" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D126" s="9"/>
       <c r="F126" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>256</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>257</v>
       </c>
+      <c r="C127" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D127" s="9"/>
       <c r="F127" t="b">
         <v>1</v>
       </c>
@@ -3562,259 +3951,373 @@
       <c r="B128" s="3" t="s">
         <v>259</v>
       </c>
+      <c r="C128" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D128" s="9"/>
       <c r="F128" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>260</v>
       </c>
       <c r="B129" s="3" t="s">
         <v>261</v>
       </c>
+      <c r="C129" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D129" s="9"/>
       <c r="F129" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>262</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>263</v>
       </c>
+      <c r="C130" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D130" s="9"/>
       <c r="F130" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>264</v>
       </c>
-      <c r="B131" s="3" t="s">
+      <c r="B131" s="5" t="s">
         <v>265</v>
       </c>
-      <c r="F131" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C131" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="D131" s="12" t="s">
+        <v>449</v>
+      </c>
+      <c r="E131" s="6"/>
+      <c r="F131" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G131" s="6"/>
+      <c r="H131" s="6"/>
+    </row>
+    <row r="132" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>266</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>267</v>
       </c>
+      <c r="C132" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D132" s="9"/>
       <c r="F132" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>268</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>269</v>
       </c>
+      <c r="C133" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D133" s="9"/>
       <c r="F133" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="75" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>270</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>271</v>
       </c>
+      <c r="C134" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="D134" s="9"/>
       <c r="F134" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>272</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>273</v>
       </c>
+      <c r="C135" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D135" s="9"/>
       <c r="F135" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="180" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:8" ht="180" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>274</v>
       </c>
-      <c r="B136" s="3" t="s">
+      <c r="B136" s="5" t="s">
         <v>275</v>
       </c>
-      <c r="F136" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C136" s="11" t="s">
+        <v>410</v>
+      </c>
+      <c r="D136" s="12" t="s">
+        <v>450</v>
+      </c>
+      <c r="E136" s="6"/>
+      <c r="F136" s="6" t="b">
+        <v>0</v>
+      </c>
+      <c r="G136" s="6"/>
+      <c r="H136" s="6"/>
+    </row>
+    <row r="137" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>276</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>277</v>
       </c>
+      <c r="C137" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D137" s="9"/>
       <c r="F137" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>278</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>279</v>
       </c>
+      <c r="C138" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D138" s="9"/>
       <c r="F138" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="240" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:8" ht="240" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>280</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>281</v>
       </c>
+      <c r="C139" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D139" s="10" t="s">
+        <v>451</v>
+      </c>
       <c r="F139" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>282</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>283</v>
       </c>
+      <c r="C140" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D140" s="9"/>
       <c r="F140" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>284</v>
       </c>
       <c r="B141" s="3" t="s">
         <v>285</v>
       </c>
+      <c r="C141" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D141" s="9"/>
       <c r="F141" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="210" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:8" ht="210" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>286</v>
       </c>
       <c r="B142" s="3" t="s">
         <v>287</v>
       </c>
+      <c r="C142" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D142" s="9"/>
       <c r="F142" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>288</v>
       </c>
-      <c r="B143" s="3" t="s">
+      <c r="B143" s="5" t="s">
         <v>289</v>
       </c>
+      <c r="C143" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="D143" s="12" t="s">
+        <v>452</v>
+      </c>
+      <c r="E143" s="6"/>
       <c r="F143" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>290</v>
       </c>
       <c r="B144" s="3" t="s">
         <v>291</v>
       </c>
+      <c r="C144" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D144" s="9"/>
       <c r="F144" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>292</v>
       </c>
       <c r="B145" s="3" t="s">
         <v>293</v>
       </c>
+      <c r="C145" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D145" s="9"/>
       <c r="F145" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>294</v>
       </c>
       <c r="B146" s="3" t="s">
         <v>295</v>
       </c>
+      <c r="C146" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D146" s="9"/>
       <c r="F146" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>296</v>
       </c>
       <c r="B147" s="3" t="s">
         <v>297</v>
       </c>
+      <c r="C147" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D147" s="9"/>
       <c r="F147" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>298</v>
       </c>
       <c r="B148" s="3" t="s">
         <v>299</v>
       </c>
+      <c r="C148" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D148" s="9"/>
       <c r="F148" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>300</v>
       </c>
       <c r="B149" s="3" t="s">
         <v>301</v>
       </c>
+      <c r="C149" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D149" s="9"/>
       <c r="F149" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>302</v>
       </c>
-      <c r="B150" s="3" t="s">
+      <c r="B150" s="5" t="s">
         <v>303</v>
       </c>
+      <c r="C150" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D150" s="12" t="s">
+        <v>453</v>
+      </c>
+      <c r="E150" s="6"/>
       <c r="F150" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>304</v>
       </c>
       <c r="B151" s="3" t="s">
         <v>305</v>
       </c>
+      <c r="C151" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D151" s="9"/>
       <c r="F151" t="b">
         <v>1</v>
       </c>
@@ -3823,31 +4326,46 @@
       <c r="A152" t="s">
         <v>306</v>
       </c>
-      <c r="B152" s="3" t="s">
+      <c r="B152" s="5" t="s">
         <v>307</v>
       </c>
+      <c r="C152" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="D152" s="12" t="s">
+        <v>454</v>
+      </c>
+      <c r="E152" s="6"/>
       <c r="F152" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>308</v>
       </c>
       <c r="B153" s="3" t="s">
         <v>309</v>
       </c>
+      <c r="C153" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D153" s="9"/>
       <c r="F153" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>310</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>311</v>
       </c>
+      <c r="C154" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D154" s="9"/>
       <c r="F154" t="b">
         <v>1</v>
       </c>
@@ -3859,17 +4377,25 @@
       <c r="B155" s="3" t="s">
         <v>313</v>
       </c>
+      <c r="C155" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D155" s="9"/>
       <c r="F155" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>314</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>315</v>
       </c>
+      <c r="C156" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D156" s="9"/>
       <c r="F156" t="b">
         <v>1</v>
       </c>
@@ -3881,6 +4407,12 @@
       <c r="B157" s="3" t="s">
         <v>317</v>
       </c>
+      <c r="C157" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="D157" s="10" t="s">
+        <v>455</v>
+      </c>
       <c r="F157" t="b">
         <v>0</v>
       </c>
@@ -3889,42 +4421,61 @@
       <c r="A158" t="s">
         <v>318</v>
       </c>
-      <c r="B158" s="3" t="s">
+      <c r="B158" s="5" t="s">
         <v>319</v>
       </c>
+      <c r="C158" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D158" s="13"/>
+      <c r="E158" s="6"/>
       <c r="F158" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>320</v>
       </c>
       <c r="B159" s="3" t="s">
         <v>321</v>
       </c>
+      <c r="C159" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D159" s="9"/>
       <c r="F159" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>322</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>323</v>
       </c>
+      <c r="C160" s="7" t="s">
+        <v>409</v>
+      </c>
+      <c r="D160" s="10" t="s">
+        <v>456</v>
+      </c>
       <c r="F160" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>324</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>325</v>
       </c>
+      <c r="C161" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D161" s="9"/>
       <c r="F161" t="b">
         <v>1</v>
       </c>
@@ -3936,6 +4487,10 @@
       <c r="B162" s="3" t="s">
         <v>327</v>
       </c>
+      <c r="C162" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D162" s="9"/>
       <c r="F162" t="b">
         <v>1</v>
       </c>
@@ -3947,6 +4502,10 @@
       <c r="B163" s="3" t="s">
         <v>329</v>
       </c>
+      <c r="C163" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D163" s="9"/>
       <c r="F163" t="b">
         <v>1</v>
       </c>
@@ -3958,11 +4517,11 @@
       <c r="B164" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="C164" t="s">
+      <c r="C164" s="7" t="s">
         <v>411</v>
       </c>
-      <c r="D164" s="3" t="s">
-        <v>420</v>
+      <c r="D164" s="10" t="s">
+        <v>457</v>
       </c>
       <c r="E164" t="b">
         <v>1</v>
@@ -3978,17 +4537,27 @@
       <c r="B165" s="3" t="s">
         <v>333</v>
       </c>
+      <c r="C165" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D165" s="10" t="s">
+        <v>458</v>
+      </c>
       <c r="F165" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>334</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>335</v>
       </c>
+      <c r="C166" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D166" s="9"/>
       <c r="F166" t="b">
         <v>1</v>
       </c>
@@ -4000,6 +4569,10 @@
       <c r="B167" s="3" t="s">
         <v>337</v>
       </c>
+      <c r="C167" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D167" s="9"/>
       <c r="F167" t="b">
         <v>1</v>
       </c>
@@ -4011,17 +4584,28 @@
       <c r="B168" s="3" t="s">
         <v>339</v>
       </c>
+      <c r="C168" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D168" s="9"/>
       <c r="F168" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>340</v>
       </c>
-      <c r="B169" s="3" t="s">
+      <c r="B169" s="14" t="s">
         <v>341</v>
       </c>
+      <c r="C169" s="15" t="s">
+        <v>412</v>
+      </c>
+      <c r="D169" s="16" t="s">
+        <v>459</v>
+      </c>
+      <c r="E169" s="17"/>
       <c r="F169" t="b">
         <v>1</v>
       </c>
@@ -4033,6 +4617,10 @@
       <c r="B170" s="3" t="s">
         <v>343</v>
       </c>
+      <c r="C170" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D170" s="9"/>
       <c r="F170" t="b">
         <v>0</v>
       </c>
@@ -4041,9 +4629,16 @@
       <c r="A171" t="s">
         <v>344</v>
       </c>
-      <c r="B171" s="3" t="s">
+      <c r="B171" s="5" t="s">
         <v>345</v>
       </c>
+      <c r="C171" s="11" t="s">
+        <v>409</v>
+      </c>
+      <c r="D171" s="12" t="s">
+        <v>460</v>
+      </c>
+      <c r="E171" s="6"/>
       <c r="F171" t="b">
         <v>0</v>
       </c>
@@ -4052,9 +4647,16 @@
       <c r="A172" t="s">
         <v>346</v>
       </c>
-      <c r="B172" s="3" t="s">
+      <c r="B172" s="5" t="s">
         <v>347</v>
       </c>
+      <c r="C172" s="11" t="s">
+        <v>412</v>
+      </c>
+      <c r="D172" s="12" t="s">
+        <v>461</v>
+      </c>
+      <c r="E172" s="6"/>
       <c r="F172" t="b">
         <v>0</v>
       </c>
@@ -4066,6 +4668,12 @@
       <c r="B173" s="3" t="s">
         <v>349</v>
       </c>
+      <c r="C173" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="D173" s="10" t="s">
+        <v>462</v>
+      </c>
       <c r="F173" t="b">
         <v>0</v>
       </c>
@@ -4077,6 +4685,10 @@
       <c r="B174" s="3" t="s">
         <v>351</v>
       </c>
+      <c r="C174" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D174" s="9"/>
       <c r="F174" t="b">
         <v>0</v>
       </c>
@@ -4088,17 +4700,27 @@
       <c r="B175" s="3" t="s">
         <v>353</v>
       </c>
+      <c r="C175" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D175" s="10" t="s">
+        <v>463</v>
+      </c>
       <c r="F175" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>354</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>355</v>
       </c>
+      <c r="C176" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D176" s="9"/>
       <c r="F176" t="b">
         <v>1</v>
       </c>
@@ -4110,17 +4732,27 @@
       <c r="B177" s="3" t="s">
         <v>357</v>
       </c>
+      <c r="C177" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D177" s="10" t="s">
+        <v>464</v>
+      </c>
       <c r="F177" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>358</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>359</v>
       </c>
+      <c r="C178" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D178" s="9"/>
       <c r="F178" t="b">
         <v>1</v>
       </c>
@@ -4132,6 +4764,10 @@
       <c r="B179" s="3" t="s">
         <v>361</v>
       </c>
+      <c r="C179" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D179" s="9"/>
       <c r="F179" t="b">
         <v>0</v>
       </c>
@@ -4140,9 +4776,16 @@
       <c r="A180" t="s">
         <v>362</v>
       </c>
-      <c r="B180" s="3" t="s">
+      <c r="B180" s="5" t="s">
         <v>363</v>
       </c>
+      <c r="C180" s="11" t="s">
+        <v>408</v>
+      </c>
+      <c r="D180" s="12" t="s">
+        <v>465</v>
+      </c>
+      <c r="E180" s="6"/>
       <c r="F180" t="b">
         <v>0</v>
       </c>
@@ -4154,39 +4797,55 @@
       <c r="B181" s="3" t="s">
         <v>365</v>
       </c>
+      <c r="C181" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D181" s="9"/>
       <c r="F181" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>366</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>367</v>
       </c>
+      <c r="C182" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D182" s="9"/>
       <c r="F182" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>368</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>369</v>
       </c>
+      <c r="C183" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D183" s="9"/>
       <c r="F183" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>370</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>371</v>
       </c>
+      <c r="C184" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D184" s="9"/>
       <c r="F184" t="b">
         <v>1</v>
       </c>
@@ -4198,17 +4857,25 @@
       <c r="B185" s="3" t="s">
         <v>373</v>
       </c>
+      <c r="C185" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D185" s="9"/>
       <c r="F185" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>374</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>375</v>
       </c>
+      <c r="C186" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D186" s="9"/>
       <c r="F186" t="b">
         <v>1</v>
       </c>
@@ -4220,6 +4887,12 @@
       <c r="B187" s="3" t="s">
         <v>377</v>
       </c>
+      <c r="C187" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D187" s="10" t="s">
+        <v>466</v>
+      </c>
       <c r="F187" t="b">
         <v>0</v>
       </c>
@@ -4231,17 +4904,25 @@
       <c r="B188" s="3" t="s">
         <v>379</v>
       </c>
+      <c r="C188" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D188" s="9"/>
       <c r="F188" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>380</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>381</v>
       </c>
+      <c r="C189" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D189" s="9"/>
       <c r="F189" t="b">
         <v>1</v>
       </c>
@@ -4253,6 +4934,12 @@
       <c r="B190" s="3" t="s">
         <v>383</v>
       </c>
+      <c r="C190" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D190" s="10" t="s">
+        <v>467</v>
+      </c>
       <c r="F190" t="b">
         <v>0</v>
       </c>
@@ -4261,9 +4948,16 @@
       <c r="A191" t="s">
         <v>384</v>
       </c>
-      <c r="B191" s="3" t="s">
+      <c r="B191" s="5" t="s">
         <v>385</v>
       </c>
+      <c r="C191" s="11" t="s">
+        <v>407</v>
+      </c>
+      <c r="D191" s="12" t="s">
+        <v>468</v>
+      </c>
+      <c r="E191" s="6"/>
       <c r="F191" t="b">
         <v>0</v>
       </c>
@@ -4275,6 +4969,10 @@
       <c r="B192" s="3" t="s">
         <v>387</v>
       </c>
+      <c r="C192" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D192" s="9"/>
       <c r="F192" t="b">
         <v>0</v>
       </c>
@@ -4286,6 +4984,10 @@
       <c r="B193" s="3" t="s">
         <v>389</v>
       </c>
+      <c r="C193" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D193" s="9"/>
       <c r="F193" t="b">
         <v>0</v>
       </c>
@@ -4297,6 +4999,10 @@
       <c r="B194" s="3" t="s">
         <v>391</v>
       </c>
+      <c r="C194" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D194" s="9"/>
       <c r="F194" t="b">
         <v>1</v>
       </c>
@@ -4308,6 +5014,10 @@
       <c r="B195" s="3" t="s">
         <v>393</v>
       </c>
+      <c r="C195" s="7" t="s">
+        <v>412</v>
+      </c>
+      <c r="D195" s="9"/>
       <c r="F195" t="b">
         <v>0</v>
       </c>
@@ -4319,6 +5029,12 @@
       <c r="B196" s="3" t="s">
         <v>395</v>
       </c>
+      <c r="C196" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D196" s="10" t="s">
+        <v>469</v>
+      </c>
       <c r="F196" t="b">
         <v>0</v>
       </c>
@@ -4330,17 +5046,25 @@
       <c r="B197" s="3" t="s">
         <v>397</v>
       </c>
+      <c r="C197" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D197" s="9"/>
       <c r="F197" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>398</v>
       </c>
-      <c r="B198" s="3" t="s">
+      <c r="B198" s="14" t="s">
         <v>399</v>
       </c>
+      <c r="C198" s="15" t="s">
+        <v>409</v>
+      </c>
+      <c r="D198" s="18"/>
       <c r="F198" t="b">
         <v>0</v>
       </c>
@@ -4352,35 +5076,47 @@
       <c r="B199" s="3" t="s">
         <v>401</v>
       </c>
+      <c r="C199" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D199" s="9"/>
       <c r="F199" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>402</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>403</v>
       </c>
+      <c r="C200" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D200" s="9"/>
       <c r="F200" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>404</v>
       </c>
       <c r="B201" s="3" t="s">
         <v>405</v>
       </c>
+      <c r="C201" s="7" t="s">
+        <v>408</v>
+      </c>
+      <c r="D201" s="9"/>
       <c r="F201" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C202:C1048576 C1">
       <formula1>$G$2:$G$7</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>